<commit_message>
Addition of Neverland example
POLIMI-TEM 2 Regions Planning Example
</commit_message>
<xml_diff>
--- a/hypatia/examples/Planning_2Regions/parameters/parameters_connections.xlsx
+++ b/hypatia/examples/Planning_2Regions/parameters/parameters_connections.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polimi365-my.sharepoint.com/personal/10776907_polimi_it/Documents/Documenti/GitHub/Hypatia-polimi/hypatia/examples/Planning_2Regions/parameters/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polimi365-my.sharepoint.com/personal/10394890_polimi_it/Documents/Research/Repositories/Hypatia-polimi/hypatia/examples/Planning_2Regions/parameters/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="11_92295E8662698944CF86836BC3D81F93A9CF84B3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8AA14C7E-E177-46DE-BB52-8360500FA2E1}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="11_92295E8662698944CF86836BC3D81F93A9CF84B3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F6DB6FE1-9150-4301-A73F-B8E2AF2685E4}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="F_OM" sheetId="1" r:id="rId1"/>
@@ -544,14 +544,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G34"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.36328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -564,7 +564,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -587,12 +587,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -615,7 +615,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -638,7 +638,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -661,7 +661,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>13</v>
       </c>
@@ -684,7 +684,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
@@ -707,7 +707,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
@@ -730,7 +730,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>16</v>
       </c>
@@ -753,7 +753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>17</v>
       </c>
@@ -776,7 +776,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>18</v>
       </c>
@@ -799,7 +799,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>19</v>
       </c>
@@ -822,7 +822,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>20</v>
       </c>
@@ -845,7 +845,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>21</v>
       </c>
@@ -868,7 +868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>22</v>
       </c>
@@ -891,7 +891,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>23</v>
       </c>
@@ -914,7 +914,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>24</v>
       </c>
@@ -937,7 +937,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>25</v>
       </c>
@@ -960,7 +960,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>26</v>
       </c>
@@ -983,7 +983,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>27</v>
       </c>
@@ -1006,7 +1006,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>28</v>
       </c>
@@ -1029,7 +1029,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>29</v>
       </c>
@@ -1052,7 +1052,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>30</v>
       </c>
@@ -1075,7 +1075,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>31</v>
       </c>
@@ -1098,7 +1098,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>32</v>
       </c>
@@ -1121,7 +1121,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>33</v>
       </c>
@@ -1144,7 +1144,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>34</v>
       </c>
@@ -1167,7 +1167,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>35</v>
       </c>
@@ -1190,7 +1190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>36</v>
       </c>
@@ -1213,7 +1213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>37</v>
       </c>
@@ -1236,7 +1236,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>38</v>
       </c>
@@ -1259,7 +1259,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>39</v>
       </c>
@@ -1282,7 +1282,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>40</v>
       </c>
@@ -1316,9 +1316,9 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1331,7 +1331,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -1354,12 +1354,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>44</v>
       </c>
@@ -1393,9 +1393,9 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1408,7 +1408,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -1431,12 +1431,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>45</v>
       </c>
@@ -1470,9 +1470,9 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:G34"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1485,7 +1485,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -1508,12 +1508,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -1536,7 +1536,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -1559,7 +1559,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -1582,7 +1582,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>13</v>
       </c>
@@ -1605,7 +1605,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
@@ -1628,7 +1628,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
@@ -1651,7 +1651,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>16</v>
       </c>
@@ -1674,7 +1674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>17</v>
       </c>
@@ -1697,7 +1697,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>18</v>
       </c>
@@ -1720,7 +1720,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>19</v>
       </c>
@@ -1743,7 +1743,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>20</v>
       </c>
@@ -1766,7 +1766,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>21</v>
       </c>
@@ -1789,7 +1789,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>22</v>
       </c>
@@ -1812,7 +1812,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>23</v>
       </c>
@@ -1835,7 +1835,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>24</v>
       </c>
@@ -1858,7 +1858,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>25</v>
       </c>
@@ -1881,7 +1881,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>26</v>
       </c>
@@ -1904,7 +1904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>27</v>
       </c>
@@ -1927,7 +1927,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>28</v>
       </c>
@@ -1950,7 +1950,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>29</v>
       </c>
@@ -1973,7 +1973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>30</v>
       </c>
@@ -1996,7 +1996,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>31</v>
       </c>
@@ -2019,7 +2019,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>32</v>
       </c>
@@ -2042,7 +2042,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>33</v>
       </c>
@@ -2065,7 +2065,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>34</v>
       </c>
@@ -2088,7 +2088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>35</v>
       </c>
@@ -2111,7 +2111,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>36</v>
       </c>
@@ -2134,7 +2134,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>37</v>
       </c>
@@ -2157,7 +2157,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>38</v>
       </c>
@@ -2180,7 +2180,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>39</v>
       </c>
@@ -2203,7 +2203,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>40</v>
       </c>
@@ -2237,9 +2237,9 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:G34"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2252,7 +2252,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -2275,12 +2275,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -2303,7 +2303,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -2326,7 +2326,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -2349,7 +2349,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>13</v>
       </c>
@@ -2372,7 +2372,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
@@ -2395,7 +2395,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
@@ -2418,7 +2418,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>16</v>
       </c>
@@ -2441,7 +2441,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>17</v>
       </c>
@@ -2464,7 +2464,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>18</v>
       </c>
@@ -2487,7 +2487,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>19</v>
       </c>
@@ -2510,7 +2510,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>20</v>
       </c>
@@ -2533,7 +2533,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>21</v>
       </c>
@@ -2556,7 +2556,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>22</v>
       </c>
@@ -2579,7 +2579,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>23</v>
       </c>
@@ -2602,7 +2602,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>24</v>
       </c>
@@ -2625,7 +2625,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>25</v>
       </c>
@@ -2648,7 +2648,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>26</v>
       </c>
@@ -2671,7 +2671,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>27</v>
       </c>
@@ -2694,7 +2694,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>28</v>
       </c>
@@ -2717,7 +2717,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>29</v>
       </c>
@@ -2740,7 +2740,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>30</v>
       </c>
@@ -2763,7 +2763,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>31</v>
       </c>
@@ -2786,7 +2786,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>32</v>
       </c>
@@ -2809,7 +2809,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>33</v>
       </c>
@@ -2832,7 +2832,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>34</v>
       </c>
@@ -2855,7 +2855,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>35</v>
       </c>
@@ -2878,7 +2878,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>36</v>
       </c>
@@ -2901,7 +2901,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>37</v>
       </c>
@@ -2924,7 +2924,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>38</v>
       </c>
@@ -2947,7 +2947,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>39</v>
       </c>
@@ -2970,7 +2970,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>40</v>
       </c>
@@ -3004,9 +3004,9 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:G34"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3019,7 +3019,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -3042,12 +3042,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -3070,7 +3070,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -3093,7 +3093,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -3116,7 +3116,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>13</v>
       </c>
@@ -3139,7 +3139,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
@@ -3162,7 +3162,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
@@ -3185,7 +3185,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>16</v>
       </c>
@@ -3208,7 +3208,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>17</v>
       </c>
@@ -3231,7 +3231,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>18</v>
       </c>
@@ -3254,7 +3254,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>19</v>
       </c>
@@ -3277,7 +3277,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>20</v>
       </c>
@@ -3300,7 +3300,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>21</v>
       </c>
@@ -3323,7 +3323,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>22</v>
       </c>
@@ -3346,7 +3346,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>23</v>
       </c>
@@ -3369,7 +3369,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>24</v>
       </c>
@@ -3392,7 +3392,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>25</v>
       </c>
@@ -3415,7 +3415,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>26</v>
       </c>
@@ -3438,7 +3438,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>27</v>
       </c>
@@ -3461,7 +3461,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>28</v>
       </c>
@@ -3484,7 +3484,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>29</v>
       </c>
@@ -3507,7 +3507,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>30</v>
       </c>
@@ -3530,7 +3530,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>31</v>
       </c>
@@ -3553,7 +3553,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>32</v>
       </c>
@@ -3576,7 +3576,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>33</v>
       </c>
@@ -3599,7 +3599,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>34</v>
       </c>
@@ -3622,7 +3622,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>35</v>
       </c>
@@ -3645,7 +3645,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>36</v>
       </c>
@@ -3668,7 +3668,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>37</v>
       </c>
@@ -3691,7 +3691,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>38</v>
       </c>
@@ -3714,7 +3714,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>39</v>
       </c>
@@ -3737,7 +3737,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>40</v>
       </c>
@@ -3771,9 +3771,9 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3786,7 +3786,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -3809,12 +3809,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>46</v>
       </c>
@@ -3848,9 +3848,9 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <dimension ref="A1:G34"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3863,7 +3863,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -3886,12 +3886,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -3914,7 +3914,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -3937,7 +3937,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -3960,7 +3960,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>13</v>
       </c>
@@ -3983,7 +3983,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
@@ -4006,7 +4006,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
@@ -4029,7 +4029,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>16</v>
       </c>
@@ -4052,7 +4052,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>17</v>
       </c>
@@ -4075,7 +4075,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>18</v>
       </c>
@@ -4098,7 +4098,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>19</v>
       </c>
@@ -4121,7 +4121,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>20</v>
       </c>
@@ -4144,7 +4144,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>21</v>
       </c>
@@ -4167,7 +4167,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>22</v>
       </c>
@@ -4190,7 +4190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>23</v>
       </c>
@@ -4213,7 +4213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>24</v>
       </c>
@@ -4236,7 +4236,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>25</v>
       </c>
@@ -4259,7 +4259,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>26</v>
       </c>
@@ -4282,7 +4282,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>27</v>
       </c>
@@ -4305,7 +4305,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>28</v>
       </c>
@@ -4328,7 +4328,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>29</v>
       </c>
@@ -4351,7 +4351,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>30</v>
       </c>
@@ -4374,7 +4374,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>31</v>
       </c>
@@ -4397,7 +4397,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>32</v>
       </c>
@@ -4420,7 +4420,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>33</v>
       </c>
@@ -4443,7 +4443,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>34</v>
       </c>
@@ -4466,7 +4466,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>35</v>
       </c>
@@ -4489,7 +4489,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>36</v>
       </c>
@@ -4512,7 +4512,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>37</v>
       </c>
@@ -4535,7 +4535,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>38</v>
       </c>
@@ -4558,7 +4558,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>39</v>
       </c>
@@ -4581,7 +4581,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>40</v>
       </c>
@@ -4615,9 +4615,9 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
   <dimension ref="A1:G34"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4630,7 +4630,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -4653,12 +4653,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -4681,7 +4681,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -4704,7 +4704,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -4727,7 +4727,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>13</v>
       </c>
@@ -4750,7 +4750,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
@@ -4773,7 +4773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
@@ -4796,7 +4796,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>16</v>
       </c>
@@ -4819,7 +4819,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>17</v>
       </c>
@@ -4842,7 +4842,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>18</v>
       </c>
@@ -4865,7 +4865,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>19</v>
       </c>
@@ -4888,7 +4888,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>20</v>
       </c>
@@ -4911,7 +4911,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>21</v>
       </c>
@@ -4934,7 +4934,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>22</v>
       </c>
@@ -4957,7 +4957,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>23</v>
       </c>
@@ -4980,7 +4980,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>24</v>
       </c>
@@ -5003,7 +5003,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>25</v>
       </c>
@@ -5026,7 +5026,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>26</v>
       </c>
@@ -5049,7 +5049,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>27</v>
       </c>
@@ -5072,7 +5072,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>28</v>
       </c>
@@ -5095,7 +5095,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>29</v>
       </c>
@@ -5118,7 +5118,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>30</v>
       </c>
@@ -5141,7 +5141,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>31</v>
       </c>
@@ -5164,7 +5164,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>32</v>
       </c>
@@ -5187,7 +5187,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>33</v>
       </c>
@@ -5210,7 +5210,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>34</v>
       </c>
@@ -5233,7 +5233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>35</v>
       </c>
@@ -5256,7 +5256,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>36</v>
       </c>
@@ -5279,7 +5279,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>37</v>
       </c>
@@ -5302,7 +5302,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>38</v>
       </c>
@@ -5325,7 +5325,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>39</v>
       </c>
@@ -5348,7 +5348,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>40</v>
       </c>
@@ -5382,9 +5382,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G34"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5397,7 +5397,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -5420,12 +5420,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -5448,7 +5448,7 @@
         <v>1.315E-4</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -5471,7 +5471,7 @@
         <v>1.315E-4</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -5494,7 +5494,7 @@
         <v>1.315E-4</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>13</v>
       </c>
@@ -5517,7 +5517,7 @@
         <v>1.315E-4</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
@@ -5540,7 +5540,7 @@
         <v>1.315E-4</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
@@ -5563,7 +5563,7 @@
         <v>1.315E-4</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>16</v>
       </c>
@@ -5586,7 +5586,7 @@
         <v>1.315E-4</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>17</v>
       </c>
@@ -5609,7 +5609,7 @@
         <v>1.315E-4</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>18</v>
       </c>
@@ -5632,7 +5632,7 @@
         <v>1.315E-4</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>19</v>
       </c>
@@ -5655,7 +5655,7 @@
         <v>1.315E-4</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>20</v>
       </c>
@@ -5678,7 +5678,7 @@
         <v>1.315E-4</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>21</v>
       </c>
@@ -5701,7 +5701,7 @@
         <v>1.315E-4</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>22</v>
       </c>
@@ -5724,7 +5724,7 @@
         <v>1.315E-4</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>23</v>
       </c>
@@ -5747,7 +5747,7 @@
         <v>1.315E-4</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>24</v>
       </c>
@@ -5770,7 +5770,7 @@
         <v>1.315E-4</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>25</v>
       </c>
@@ -5793,7 +5793,7 @@
         <v>1.315E-4</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>26</v>
       </c>
@@ -5816,7 +5816,7 @@
         <v>1.315E-4</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>27</v>
       </c>
@@ -5839,7 +5839,7 @@
         <v>1.315E-4</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>28</v>
       </c>
@@ -5862,7 +5862,7 @@
         <v>1.315E-4</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>29</v>
       </c>
@@ -5885,7 +5885,7 @@
         <v>1.315E-4</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>30</v>
       </c>
@@ -5908,7 +5908,7 @@
         <v>1.315E-4</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>31</v>
       </c>
@@ -5931,7 +5931,7 @@
         <v>1.315E-4</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>32</v>
       </c>
@@ -5954,7 +5954,7 @@
         <v>1.315E-4</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>33</v>
       </c>
@@ -5977,7 +5977,7 @@
         <v>1.315E-4</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>34</v>
       </c>
@@ -6000,7 +6000,7 @@
         <v>1.315E-4</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>35</v>
       </c>
@@ -6023,7 +6023,7 @@
         <v>1.315E-4</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>36</v>
       </c>
@@ -6046,7 +6046,7 @@
         <v>1.315E-4</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>37</v>
       </c>
@@ -6069,7 +6069,7 @@
         <v>1.315E-4</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>38</v>
       </c>
@@ -6092,7 +6092,7 @@
         <v>1.315E-4</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>39</v>
       </c>
@@ -6115,7 +6115,7 @@
         <v>1.315E-4</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>40</v>
       </c>
@@ -6149,9 +6149,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G34"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="7" max="7" width="13.90625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6164,7 +6167,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -6187,12 +6190,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -6215,7 +6218,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -6238,7 +6241,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -6261,7 +6264,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>13</v>
       </c>
@@ -6284,7 +6287,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
@@ -6307,7 +6310,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
@@ -6330,7 +6333,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>16</v>
       </c>
@@ -6353,7 +6356,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>17</v>
       </c>
@@ -6376,7 +6379,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>18</v>
       </c>
@@ -6399,7 +6402,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>19</v>
       </c>
@@ -6422,7 +6425,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>20</v>
       </c>
@@ -6445,7 +6448,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>21</v>
       </c>
@@ -6468,7 +6471,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>22</v>
       </c>
@@ -6491,7 +6494,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>23</v>
       </c>
@@ -6514,7 +6517,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>24</v>
       </c>
@@ -6537,7 +6540,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>25</v>
       </c>
@@ -6560,7 +6563,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>26</v>
       </c>
@@ -6583,7 +6586,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>27</v>
       </c>
@@ -6606,7 +6609,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>28</v>
       </c>
@@ -6629,7 +6632,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>29</v>
       </c>
@@ -6652,7 +6655,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>30</v>
       </c>
@@ -6675,7 +6678,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>31</v>
       </c>
@@ -6698,7 +6701,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>32</v>
       </c>
@@ -6721,7 +6724,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>33</v>
       </c>
@@ -6744,7 +6747,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>34</v>
       </c>
@@ -6767,7 +6770,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>35</v>
       </c>
@@ -6790,7 +6793,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>36</v>
       </c>
@@ -6813,7 +6816,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>37</v>
       </c>
@@ -6836,7 +6839,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>38</v>
       </c>
@@ -6859,7 +6862,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>39</v>
       </c>
@@ -6882,7 +6885,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>40</v>
       </c>
@@ -6916,9 +6919,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:G34"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="7" max="7" width="13.90625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6931,7 +6937,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -6954,12 +6960,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -6982,7 +6988,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -7005,7 +7011,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -7028,7 +7034,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>13</v>
       </c>
@@ -7051,7 +7057,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
@@ -7074,7 +7080,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
@@ -7097,7 +7103,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>16</v>
       </c>
@@ -7120,7 +7126,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>17</v>
       </c>
@@ -7143,7 +7149,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>18</v>
       </c>
@@ -7166,7 +7172,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>19</v>
       </c>
@@ -7189,7 +7195,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>20</v>
       </c>
@@ -7212,7 +7218,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>21</v>
       </c>
@@ -7235,7 +7241,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>22</v>
       </c>
@@ -7258,7 +7264,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>23</v>
       </c>
@@ -7281,7 +7287,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>24</v>
       </c>
@@ -7304,7 +7310,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>25</v>
       </c>
@@ -7327,7 +7333,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>26</v>
       </c>
@@ -7350,7 +7356,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>27</v>
       </c>
@@ -7373,7 +7379,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>28</v>
       </c>
@@ -7396,7 +7402,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>29</v>
       </c>
@@ -7419,7 +7425,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>30</v>
       </c>
@@ -7442,7 +7448,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>31</v>
       </c>
@@ -7465,7 +7471,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>32</v>
       </c>
@@ -7488,7 +7494,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>33</v>
       </c>
@@ -7511,7 +7517,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>34</v>
       </c>
@@ -7534,7 +7540,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>35</v>
       </c>
@@ -7557,7 +7563,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>36</v>
       </c>
@@ -7580,7 +7586,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>37</v>
       </c>
@@ -7603,7 +7609,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>38</v>
       </c>
@@ -7626,7 +7632,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>39</v>
       </c>
@@ -7649,7 +7655,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>40</v>
       </c>
@@ -7683,9 +7689,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:G34"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="7" max="7" width="13.90625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -7698,7 +7707,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -7721,12 +7730,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -7749,7 +7758,7 @@
         <v>124.77</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -7772,7 +7781,7 @@
         <v>124.77</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -7795,7 +7804,7 @@
         <v>124.77</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>13</v>
       </c>
@@ -7818,7 +7827,7 @@
         <v>124.77</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
@@ -7841,7 +7850,7 @@
         <v>124.77</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
@@ -7864,7 +7873,7 @@
         <v>124.77</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>16</v>
       </c>
@@ -7887,7 +7896,7 @@
         <v>124.77</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>17</v>
       </c>
@@ -7910,7 +7919,7 @@
         <v>124.77</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>18</v>
       </c>
@@ -7933,7 +7942,7 @@
         <v>124.77</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>19</v>
       </c>
@@ -7956,7 +7965,7 @@
         <v>124.77</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>20</v>
       </c>
@@ -7979,7 +7988,7 @@
         <v>124.77</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>21</v>
       </c>
@@ -8002,7 +8011,7 @@
         <v>124.77</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>22</v>
       </c>
@@ -8025,7 +8034,7 @@
         <v>124.77</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>23</v>
       </c>
@@ -8048,7 +8057,7 @@
         <v>124.77</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>24</v>
       </c>
@@ -8071,7 +8080,7 @@
         <v>124.77</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>25</v>
       </c>
@@ -8094,7 +8103,7 @@
         <v>124.77</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>26</v>
       </c>
@@ -8117,7 +8126,7 @@
         <v>124.77</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>27</v>
       </c>
@@ -8140,7 +8149,7 @@
         <v>124.77</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>28</v>
       </c>
@@ -8163,7 +8172,7 @@
         <v>124.77</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>29</v>
       </c>
@@ -8186,7 +8195,7 @@
         <v>124.77</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>30</v>
       </c>
@@ -8209,7 +8218,7 @@
         <v>124.77</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>31</v>
       </c>
@@ -8232,7 +8241,7 @@
         <v>124.77</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>32</v>
       </c>
@@ -8255,7 +8264,7 @@
         <v>124.77</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>33</v>
       </c>
@@ -8278,7 +8287,7 @@
         <v>124.77</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>34</v>
       </c>
@@ -8301,7 +8310,7 @@
         <v>124.77</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>35</v>
       </c>
@@ -8324,7 +8333,7 @@
         <v>124.77</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>36</v>
       </c>
@@ -8347,7 +8356,7 @@
         <v>124.77</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>37</v>
       </c>
@@ -8370,7 +8379,7 @@
         <v>124.77</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>38</v>
       </c>
@@ -8393,7 +8402,7 @@
         <v>124.77</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>39</v>
       </c>
@@ -8416,7 +8425,7 @@
         <v>124.77</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>40</v>
       </c>
@@ -8450,9 +8459,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:G34"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -8465,7 +8474,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -8488,12 +8497,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -8516,7 +8525,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -8539,7 +8548,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -8562,7 +8571,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>13</v>
       </c>
@@ -8585,7 +8594,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
@@ -8608,7 +8617,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
@@ -8631,7 +8640,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>16</v>
       </c>
@@ -8654,7 +8663,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>17</v>
       </c>
@@ -8677,7 +8686,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>18</v>
       </c>
@@ -8700,7 +8709,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>19</v>
       </c>
@@ -8723,7 +8732,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>20</v>
       </c>
@@ -8746,7 +8755,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>21</v>
       </c>
@@ -8769,7 +8778,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>22</v>
       </c>
@@ -8792,7 +8801,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>23</v>
       </c>
@@ -8815,7 +8824,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>24</v>
       </c>
@@ -8838,7 +8847,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>25</v>
       </c>
@@ -8861,7 +8870,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>26</v>
       </c>
@@ -8884,7 +8893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>27</v>
       </c>
@@ -8907,7 +8916,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>28</v>
       </c>
@@ -8930,7 +8939,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>29</v>
       </c>
@@ -8953,7 +8962,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>30</v>
       </c>
@@ -8976,7 +8985,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>31</v>
       </c>
@@ -8999,7 +9008,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>32</v>
       </c>
@@ -9022,7 +9031,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>33</v>
       </c>
@@ -9045,7 +9054,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>34</v>
       </c>
@@ -9068,7 +9077,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>35</v>
       </c>
@@ -9091,7 +9100,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>36</v>
       </c>
@@ -9114,7 +9123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>37</v>
       </c>
@@ -9137,7 +9146,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>38</v>
       </c>
@@ -9160,7 +9169,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>39</v>
       </c>
@@ -9183,7 +9192,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>40</v>
       </c>
@@ -9217,9 +9226,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:G34"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -9232,7 +9241,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -9255,12 +9264,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -9283,7 +9292,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -9306,7 +9315,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -9329,7 +9338,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>13</v>
       </c>
@@ -9352,7 +9361,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
@@ -9375,7 +9384,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
@@ -9398,7 +9407,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>16</v>
       </c>
@@ -9421,7 +9430,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>17</v>
       </c>
@@ -9444,7 +9453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>18</v>
       </c>
@@ -9467,7 +9476,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>19</v>
       </c>
@@ -9490,7 +9499,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>20</v>
       </c>
@@ -9513,7 +9522,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>21</v>
       </c>
@@ -9536,7 +9545,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>22</v>
       </c>
@@ -9559,7 +9568,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>23</v>
       </c>
@@ -9582,7 +9591,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>24</v>
       </c>
@@ -9605,7 +9614,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>25</v>
       </c>
@@ -9628,7 +9637,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>26</v>
       </c>
@@ -9651,7 +9660,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>27</v>
       </c>
@@ -9674,7 +9683,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>28</v>
       </c>
@@ -9697,7 +9706,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>29</v>
       </c>
@@ -9720,7 +9729,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>30</v>
       </c>
@@ -9743,7 +9752,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>31</v>
       </c>
@@ -9766,7 +9775,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>32</v>
       </c>
@@ -9789,7 +9798,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>33</v>
       </c>
@@ -9812,7 +9821,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>34</v>
       </c>
@@ -9835,7 +9844,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>35</v>
       </c>
@@ -9858,7 +9867,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>36</v>
       </c>
@@ -9881,7 +9890,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>37</v>
       </c>
@@ -9904,7 +9913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>38</v>
       </c>
@@ -9927,7 +9936,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>39</v>
       </c>
@@ -9950,7 +9959,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>40</v>
       </c>
@@ -9984,9 +9993,9 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -9999,7 +10008,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -10022,12 +10031,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>42</v>
       </c>
@@ -10061,9 +10070,9 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -10076,7 +10085,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -10099,12 +10108,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>43</v>
       </c>
@@ -10136,6 +10145,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100241E96938535DD4B921FCDFB54345D30" ma:contentTypeVersion="16" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="ea9f1ad5a580c8ec0c54747f8c275290">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5d44ae6a-e145-4c9d-94e7-ddf9cc58067e" xmlns:ns3="e67e9a88-35e1-4b39-8da9-a609eb308282" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0a21d2b210d3c14c0eb20b1c12c2a17c" ns2:_="" ns3:_="">
     <xsd:import namespace="5d44ae6a-e145-4c9d-94e7-ddf9cc58067e"/>
@@ -10378,16 +10396,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148490FD-B3B3-4423-BD45-D0B0893FE1B9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{362B819E-0024-4B0B-ACB7-796FEC865E82}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -10404,12 +10421,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148490FD-B3B3-4423-BD45-D0B0893FE1B9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>